<commit_message>
frekansiyel rapor excel - template yapısı güncellendi
- Giriş: Proje satırı eklendi (row 3)
- Kayıp Frekanslar: KAYIP NEDENİ kolonu (G) eklendi
- Gruplar: GÖREV TANIMI kolonu kaldırıldı (10 kolon)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/report-templates/QR-SYNC_Genel_Rapor.xlsx
+++ b/public/report-templates/QR-SYNC_Genel_Rapor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giriş" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tamamlanan Frekanslar" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sapmalar" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kayıp Frekanslar" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruplar" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Giriş" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tamamlanan Frekanslar" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sapmalar" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Kayıp Frekanslar" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruplar" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tamamlanan Frekanslar'!$A$2:$E$8</definedName>
@@ -27,7 +27,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="&quot;₺&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -148,8 +148,13 @@
       <sz val="12"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -180,6 +185,11 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="52">
     <border>
@@ -803,7 +813,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1306,6 +1316,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="51" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1397,14 +1410,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -1441,16 +1454,16 @@
       </layout>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -1493,10 +1506,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:schemeClr val="accent1"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1504,18 +1517,18 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1200" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1581,8 +1594,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -1594,9 +1607,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1050" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1632,7 +1645,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -1649,16 +1662,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+          <a:ln>
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1400" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1687,10 +1700,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -1705,7 +1718,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -1740,7 +1753,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:pattFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="narHorz">
+            <a:pattFill prst="narHorz">
               <a:fgClr>
                 <a:schemeClr val="accent1"/>
               </a:fgClr>
@@ -1751,7 +1764,7 @@
                 </a:schemeClr>
               </a:bgClr>
             </a:pattFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -1759,18 +1772,18 @@
           <invertIfNegative val="0"/>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -1834,8 +1847,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill/>
+          <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="25000"/>
@@ -1847,9 +1860,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1888,16 +1901,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+          <a:ln>
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1050" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -1927,16 +1940,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -1961,8 +1974,8 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:noFill/>
       <a:prstDash val="solid"/>
       <a:round/>
@@ -1972,13 +1985,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="1"/>
             </a:pPr>
@@ -1992,16 +2005,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -2041,7 +2054,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -2049,10 +2062,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2062,10 +2075,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2083,18 +2096,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1100" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2164,16 +2177,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -2198,10 +2211,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -2216,14 +2229,14 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -2252,16 +2265,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -2292,10 +2305,10 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:schemeClr val="accent1"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
@@ -2306,10 +2319,10 @@
             <invertIfNegative val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="00B0F0"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2320,10 +2333,10 @@
             <invertIfNegative val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="00B050"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2334,13 +2347,13 @@
             <invertIfNegative val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent2">
                   <a:lumMod val="40000"/>
                   <a:lumOff val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2351,12 +2364,12 @@
             <invertIfNegative val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="bg2">
                   <a:lumMod val="75000"/>
                 </a:schemeClr>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2364,18 +2377,18 @@
           </dPt>
           <dLbls>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="1050" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2463,8 +2476,8 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
               <a:schemeClr val="tx1">
                 <a:lumMod val="15000"/>
@@ -2476,9 +2489,9 @@
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2514,7 +2527,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="15000"/>
@@ -2531,16 +2544,16 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:noFill/>
+          <a:ln>
             <a:noFill/>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
@@ -2569,10 +2582,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -2587,14 +2600,14 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr>
               <a:defRPr sz="1200" b="1" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
                 <a:solidFill>
@@ -2619,16 +2632,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1200" b="0" i="0" strike="noStrike" kern="1200" spc="0" baseline="0">
               <a:solidFill>
@@ -2668,7 +2681,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -2676,10 +2689,10 @@
             <idx val="0"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2689,10 +2702,10 @@
             <idx val="1"/>
             <bubble3D val="0"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
@@ -2702,18 +2715,18 @@
             <dLbl>
               <idx val="0"/>
               <spPr>
-                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:ln>
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1100" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -2744,18 +2757,18 @@
             <dLbl>
               <idx val="1"/>
               <spPr>
-                <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:noFill/>
+                <a:ln>
                   <a:noFill/>
                   <a:prstDash val="solid"/>
                 </a:ln>
               </spPr>
               <txPr>
-                <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                   <a:spAutoFit/>
                 </a:bodyPr>
-                <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-                <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:lstStyle/>
+                <a:p>
                   <a:pPr>
                     <a:defRPr sz="1100" b="1" i="0" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
@@ -2784,18 +2797,18 @@
               <showBubbleSize val="0"/>
             </dLbl>
             <spPr>
-              <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:noFill/>
+              <a:ln>
                 <a:noFill/>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
             <txPr>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
                 <a:spAutoFit/>
               </a:bodyPr>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr sz="900" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
@@ -2866,16 +2879,16 @@
       <layout/>
       <overlay val="0"/>
       <spPr>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:noFill/>
+        <a:ln>
           <a:noFill/>
           <a:prstDash val="solid"/>
         </a:ln>
       </spPr>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr>
             <a:defRPr sz="1100" b="0" i="0" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
@@ -2900,10 +2913,10 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+    <a:solidFill>
       <a:schemeClr val="bg1"/>
     </a:solidFill>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525" cap="flat" cmpd="sng" algn="ctr">
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
       <a:solidFill>
         <a:schemeClr val="tx1">
           <a:lumMod val="15000"/>
@@ -2918,7 +2931,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>1</col>
@@ -2938,9 +2951,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2965,9 +2978,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2992,9 +3005,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3019,9 +3032,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3046,9 +3059,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -3324,7 +3337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:BR30"/>
+  <dimension ref="A1:BR31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="2.6640625" customWidth="1" style="42" min="1" max="1"/>
@@ -3422,88 +3435,23 @@
       <c r="BP2" s="7" t="n"/>
     </row>
     <row r="3" ht="31.8" customHeight="1" s="42">
-      <c r="B3" s="156" t="n"/>
-      <c r="C3" s="157" t="inlineStr">
-        <is>
-          <t>Üst Lokasyon:</t>
-        </is>
-      </c>
-      <c r="D3" s="158" t="n"/>
-      <c r="E3" s="158" t="n"/>
-      <c r="F3" s="159" t="n"/>
-      <c r="G3" s="93" t="n"/>
-      <c r="H3" s="158" t="n"/>
-      <c r="I3" s="158" t="n"/>
-      <c r="J3" s="158" t="n"/>
-      <c r="K3" s="158" t="n"/>
-      <c r="L3" s="158" t="n"/>
-      <c r="M3" s="158" t="n"/>
-      <c r="N3" s="158" t="n"/>
-      <c r="O3" s="158" t="n"/>
-      <c r="P3" s="159" t="n"/>
-      <c r="S3" s="57" t="n"/>
-      <c r="T3" s="56" t="n"/>
-      <c r="Z3" s="57" t="n"/>
-      <c r="AQ3" s="67" t="inlineStr">
-        <is>
-          <t>GRUP TANIMI</t>
-        </is>
-      </c>
-      <c r="AR3" s="158" t="n"/>
-      <c r="AS3" s="158" t="n"/>
-      <c r="AT3" s="158" t="n"/>
-      <c r="AU3" s="159" t="n"/>
-      <c r="AV3" s="74" t="inlineStr">
-        <is>
-          <t>HEDEF FREKANS</t>
-        </is>
-      </c>
-      <c r="AW3" s="158" t="n"/>
-      <c r="AX3" s="158" t="n"/>
-      <c r="AY3" s="159" t="n"/>
-      <c r="AZ3" s="74" t="inlineStr">
-        <is>
-          <t>BİRİM FİYAT</t>
-        </is>
-      </c>
-      <c r="BA3" s="158" t="n"/>
-      <c r="BB3" s="159" t="n"/>
-      <c r="BC3" s="74" t="inlineStr">
-        <is>
-          <t>TOPLAM HAKEDİŞ</t>
-        </is>
-      </c>
-      <c r="BD3" s="158" t="n"/>
-      <c r="BE3" s="158" t="n"/>
-      <c r="BF3" s="159" t="n"/>
-      <c r="BG3" s="74" t="inlineStr">
-        <is>
-          <t>KAYIP FREKANS</t>
-        </is>
-      </c>
-      <c r="BH3" s="158" t="n"/>
-      <c r="BI3" s="159" t="n"/>
-      <c r="BJ3" s="74" t="inlineStr">
-        <is>
-          <t>KAYIP HAKEDİŞ</t>
-        </is>
-      </c>
-      <c r="BK3" s="158" t="n"/>
-      <c r="BL3" s="159" t="n"/>
-      <c r="BM3" s="128" t="inlineStr">
-        <is>
-          <t>GERÇEKLEŞEN HAKEDİŞ</t>
-        </is>
-      </c>
-      <c r="BN3" s="158" t="n"/>
-      <c r="BO3" s="158" t="n"/>
-      <c r="BP3" s="160" t="n"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Proje</t>
+        </is>
+      </c>
+      <c r="B3" s="151" t="n"/>
+      <c r="C3" s="152" t="n"/>
+      <c r="D3" s="153" t="n"/>
+      <c r="E3" s="153" t="n"/>
+      <c r="F3" s="154" t="n"/>
+      <c r="G3" s="97" t="inlineStr"/>
     </row>
     <row r="4" ht="20.4" customHeight="1" s="42">
       <c r="B4" s="156" t="n"/>
       <c r="C4" s="157" t="inlineStr">
         <is>
-          <t>Alt Lokasyon</t>
+          <t>Üst Lokasyon:</t>
         </is>
       </c>
       <c r="D4" s="158" t="n"/>
@@ -3522,29 +3470,57 @@
       <c r="S4" s="57" t="n"/>
       <c r="T4" s="56" t="n"/>
       <c r="Z4" s="57" t="n"/>
-      <c r="AQ4" s="67" t="n"/>
+      <c r="AQ4" s="67" t="inlineStr">
+        <is>
+          <t>GRUP TANIMI</t>
+        </is>
+      </c>
       <c r="AR4" s="158" t="n"/>
       <c r="AS4" s="158" t="n"/>
       <c r="AT4" s="158" t="n"/>
       <c r="AU4" s="159" t="n"/>
-      <c r="AV4" s="111" t="n"/>
+      <c r="AV4" s="74" t="inlineStr">
+        <is>
+          <t>HEDEF FREKANS</t>
+        </is>
+      </c>
       <c r="AW4" s="158" t="n"/>
       <c r="AX4" s="158" t="n"/>
       <c r="AY4" s="159" t="n"/>
-      <c r="AZ4" s="161" t="n"/>
+      <c r="AZ4" s="74" t="inlineStr">
+        <is>
+          <t>BİRİM FİYAT</t>
+        </is>
+      </c>
       <c r="BA4" s="158" t="n"/>
       <c r="BB4" s="159" t="n"/>
-      <c r="BC4" s="162" t="n"/>
+      <c r="BC4" s="74" t="inlineStr">
+        <is>
+          <t>TOPLAM HAKEDİŞ</t>
+        </is>
+      </c>
       <c r="BD4" s="158" t="n"/>
       <c r="BE4" s="158" t="n"/>
       <c r="BF4" s="159" t="n"/>
-      <c r="BG4" s="58" t="n"/>
+      <c r="BG4" s="74" t="inlineStr">
+        <is>
+          <t>KAYIP FREKANS</t>
+        </is>
+      </c>
       <c r="BH4" s="158" t="n"/>
       <c r="BI4" s="159" t="n"/>
-      <c r="BJ4" s="163" t="n"/>
+      <c r="BJ4" s="74" t="inlineStr">
+        <is>
+          <t>KAYIP HAKEDİŞ</t>
+        </is>
+      </c>
       <c r="BK4" s="158" t="n"/>
-      <c r="BL4" s="160" t="n"/>
-      <c r="BM4" s="164" t="n"/>
+      <c r="BL4" s="159" t="n"/>
+      <c r="BM4" s="128" t="inlineStr">
+        <is>
+          <t>GERÇEKLEŞEN HAKEDİŞ</t>
+        </is>
+      </c>
       <c r="BN4" s="158" t="n"/>
       <c r="BO4" s="158" t="n"/>
       <c r="BP4" s="160" t="n"/>
@@ -3553,7 +3529,7 @@
       <c r="B5" s="156" t="n"/>
       <c r="C5" s="157" t="inlineStr">
         <is>
-          <t>RaporTarihi:</t>
+          <t>Alt Lokasyon</t>
         </is>
       </c>
       <c r="D5" s="158" t="n"/>
@@ -3603,7 +3579,7 @@
       <c r="B6" s="156" t="n"/>
       <c r="C6" s="157" t="inlineStr">
         <is>
-          <t>Rapor Gün Sayısı:</t>
+          <t>RaporTarihi:</t>
         </is>
       </c>
       <c r="D6" s="158" t="n"/>
@@ -3650,25 +3626,25 @@
       <c r="BP6" s="160" t="n"/>
     </row>
     <row r="7" ht="20.4" customHeight="1" s="42" thickBot="1">
-      <c r="B7" s="165" t="n"/>
-      <c r="C7" s="166" t="inlineStr">
-        <is>
-          <t>Raporu Alan:</t>
-        </is>
-      </c>
-      <c r="D7" s="167" t="n"/>
-      <c r="E7" s="167" t="n"/>
-      <c r="F7" s="168" t="n"/>
-      <c r="G7" s="95" t="n"/>
-      <c r="H7" s="167" t="n"/>
-      <c r="I7" s="167" t="n"/>
-      <c r="J7" s="167" t="n"/>
-      <c r="K7" s="167" t="n"/>
-      <c r="L7" s="167" t="n"/>
-      <c r="M7" s="167" t="n"/>
-      <c r="N7" s="167" t="n"/>
-      <c r="O7" s="167" t="n"/>
-      <c r="P7" s="168" t="n"/>
+      <c r="B7" s="156" t="n"/>
+      <c r="C7" s="157" t="inlineStr">
+        <is>
+          <t>Rapor Gün Sayısı:</t>
+        </is>
+      </c>
+      <c r="D7" s="158" t="n"/>
+      <c r="E7" s="158" t="n"/>
+      <c r="F7" s="159" t="n"/>
+      <c r="G7" s="93" t="n"/>
+      <c r="H7" s="158" t="n"/>
+      <c r="I7" s="158" t="n"/>
+      <c r="J7" s="158" t="n"/>
+      <c r="K7" s="158" t="n"/>
+      <c r="L7" s="158" t="n"/>
+      <c r="M7" s="158" t="n"/>
+      <c r="N7" s="158" t="n"/>
+      <c r="O7" s="158" t="n"/>
+      <c r="P7" s="159" t="n"/>
       <c r="S7" s="57" t="n"/>
       <c r="T7" s="56" t="n"/>
       <c r="Z7" s="57" t="n"/>
@@ -3700,348 +3676,315 @@
       <c r="BP7" s="160" t="n"/>
     </row>
     <row r="8" ht="20.4" customHeight="1" s="42" thickBot="1">
+      <c r="B8" s="165" t="n"/>
+      <c r="C8" s="166" t="inlineStr">
+        <is>
+          <t>Raporu Alan:</t>
+        </is>
+      </c>
+      <c r="D8" s="167" t="n"/>
+      <c r="E8" s="167" t="n"/>
+      <c r="F8" s="168" t="n"/>
+      <c r="G8" s="95" t="n"/>
+      <c r="H8" s="167" t="n"/>
+      <c r="I8" s="167" t="n"/>
+      <c r="J8" s="167" t="n"/>
+      <c r="K8" s="167" t="n"/>
+      <c r="L8" s="167" t="n"/>
+      <c r="M8" s="167" t="n"/>
+      <c r="N8" s="167" t="n"/>
+      <c r="O8" s="167" t="n"/>
+      <c r="P8" s="168" t="n"/>
       <c r="S8" s="57" t="n"/>
       <c r="T8" s="56" t="n"/>
       <c r="Z8" s="57" t="n"/>
-      <c r="AQ8" s="141" t="n"/>
-      <c r="AR8" s="167" t="n"/>
-      <c r="AS8" s="167" t="n"/>
-      <c r="AT8" s="167" t="n"/>
-      <c r="AU8" s="168" t="n"/>
-      <c r="AV8" s="112" t="n"/>
-      <c r="AW8" s="167" t="n"/>
-      <c r="AX8" s="167" t="n"/>
-      <c r="AY8" s="168" t="n"/>
-      <c r="AZ8" s="169" t="n"/>
-      <c r="BA8" s="167" t="n"/>
-      <c r="BB8" s="168" t="n"/>
-      <c r="BC8" s="170" t="n"/>
-      <c r="BD8" s="167" t="n"/>
-      <c r="BE8" s="167" t="n"/>
-      <c r="BF8" s="168" t="n"/>
-      <c r="BG8" s="171" t="n"/>
-      <c r="BH8" s="167" t="n"/>
-      <c r="BI8" s="168" t="n"/>
-      <c r="BJ8" s="172" t="n"/>
-      <c r="BK8" s="167" t="n"/>
-      <c r="BL8" s="173" t="n"/>
-      <c r="BM8" s="174" t="n"/>
-      <c r="BN8" s="167" t="n"/>
-      <c r="BO8" s="167" t="n"/>
-      <c r="BP8" s="173" t="n"/>
+      <c r="AQ8" s="67" t="n"/>
+      <c r="AR8" s="158" t="n"/>
+      <c r="AS8" s="158" t="n"/>
+      <c r="AT8" s="158" t="n"/>
+      <c r="AU8" s="159" t="n"/>
+      <c r="AV8" s="111" t="n"/>
+      <c r="AW8" s="158" t="n"/>
+      <c r="AX8" s="158" t="n"/>
+      <c r="AY8" s="159" t="n"/>
+      <c r="AZ8" s="161" t="n"/>
+      <c r="BA8" s="158" t="n"/>
+      <c r="BB8" s="159" t="n"/>
+      <c r="BC8" s="162" t="n"/>
+      <c r="BD8" s="158" t="n"/>
+      <c r="BE8" s="158" t="n"/>
+      <c r="BF8" s="159" t="n"/>
+      <c r="BG8" s="58" t="n"/>
+      <c r="BH8" s="158" t="n"/>
+      <c r="BI8" s="159" t="n"/>
+      <c r="BJ8" s="163" t="n"/>
+      <c r="BK8" s="158" t="n"/>
+      <c r="BL8" s="160" t="n"/>
+      <c r="BM8" s="164" t="n"/>
+      <c r="BN8" s="158" t="n"/>
+      <c r="BO8" s="158" t="n"/>
+      <c r="BP8" s="160" t="n"/>
     </row>
     <row r="9" ht="7.95" customHeight="1" s="42" thickBot="1">
-      <c r="B9" s="3" t="n"/>
-      <c r="C9" s="3" t="n"/>
-      <c r="D9" s="3" t="n"/>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
-      <c r="G9" s="4" t="n"/>
-      <c r="H9" s="4" t="n"/>
-      <c r="I9" s="4" t="n"/>
-      <c r="J9" s="4" t="n"/>
-      <c r="K9" s="4" t="n"/>
-      <c r="L9" s="4" t="n"/>
-      <c r="M9" s="4" t="n"/>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4" t="n"/>
-      <c r="P9" s="4" t="n"/>
       <c r="S9" s="57" t="n"/>
       <c r="T9" s="56" t="n"/>
       <c r="Z9" s="57" t="n"/>
+      <c r="AQ9" s="141" t="n"/>
+      <c r="AR9" s="167" t="n"/>
+      <c r="AS9" s="167" t="n"/>
+      <c r="AT9" s="167" t="n"/>
+      <c r="AU9" s="168" t="n"/>
+      <c r="AV9" s="112" t="n"/>
+      <c r="AW9" s="167" t="n"/>
+      <c r="AX9" s="167" t="n"/>
+      <c r="AY9" s="168" t="n"/>
+      <c r="AZ9" s="169" t="n"/>
+      <c r="BA9" s="167" t="n"/>
+      <c r="BB9" s="168" t="n"/>
+      <c r="BC9" s="170" t="n"/>
+      <c r="BD9" s="167" t="n"/>
+      <c r="BE9" s="167" t="n"/>
+      <c r="BF9" s="168" t="n"/>
+      <c r="BG9" s="171" t="n"/>
+      <c r="BH9" s="167" t="n"/>
+      <c r="BI9" s="168" t="n"/>
+      <c r="BJ9" s="172" t="n"/>
+      <c r="BK9" s="167" t="n"/>
+      <c r="BL9" s="173" t="n"/>
+      <c r="BM9" s="174" t="n"/>
+      <c r="BN9" s="167" t="n"/>
+      <c r="BO9" s="167" t="n"/>
+      <c r="BP9" s="173" t="n"/>
     </row>
     <row r="10" ht="7.95" customHeight="1" s="42">
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="n"/>
-      <c r="K10" s="6" t="n"/>
-      <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6" t="n"/>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6" t="n"/>
-      <c r="P10" s="6" t="n"/>
-      <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="6" t="n"/>
-      <c r="S10" s="6" t="n"/>
-      <c r="T10" s="6" t="n"/>
-      <c r="U10" s="6" t="n"/>
-      <c r="V10" s="6" t="n"/>
-      <c r="W10" s="6" t="n"/>
-      <c r="X10" s="6" t="n"/>
-      <c r="Y10" s="6" t="n"/>
-      <c r="Z10" s="6" t="n"/>
-      <c r="AA10" s="6" t="n"/>
-      <c r="AB10" s="6" t="n"/>
-      <c r="AC10" s="6" t="n"/>
-      <c r="AD10" s="6" t="n"/>
-      <c r="AE10" s="6" t="n"/>
-      <c r="AF10" s="6" t="n"/>
-      <c r="AG10" s="6" t="n"/>
-      <c r="AH10" s="6" t="n"/>
-      <c r="AI10" s="6" t="n"/>
-      <c r="AJ10" s="6" t="n"/>
-      <c r="AK10" s="6" t="n"/>
-      <c r="AL10" s="6" t="n"/>
-      <c r="AM10" s="6" t="n"/>
-      <c r="AN10" s="6" t="n"/>
-      <c r="AO10" s="6" t="n"/>
-      <c r="AP10" s="6" t="n"/>
-      <c r="AQ10" s="6" t="n"/>
-      <c r="AR10" s="6" t="n"/>
-      <c r="AS10" s="6" t="n"/>
-      <c r="AT10" s="6" t="n"/>
-      <c r="AU10" s="6" t="n"/>
-      <c r="AV10" s="6" t="n"/>
-      <c r="AW10" s="6" t="n"/>
-      <c r="AX10" s="6" t="n"/>
-      <c r="AY10" s="6" t="n"/>
-      <c r="AZ10" s="6" t="n"/>
-      <c r="BA10" s="6" t="n"/>
-      <c r="BB10" s="6" t="n"/>
-      <c r="BC10" s="6" t="n"/>
-      <c r="BD10" s="6" t="n"/>
-      <c r="BE10" s="6" t="n"/>
-      <c r="BF10" s="6" t="n"/>
-      <c r="BG10" s="6" t="n"/>
-      <c r="BH10" s="6" t="n"/>
-      <c r="BI10" s="6" t="n"/>
-      <c r="BJ10" s="6" t="n"/>
-      <c r="BK10" s="6" t="n"/>
-      <c r="BL10" s="6" t="n"/>
-      <c r="BM10" s="6" t="n"/>
-      <c r="BN10" s="6" t="n"/>
-      <c r="BO10" s="6" t="n"/>
-      <c r="BP10" s="7" t="n"/>
+      <c r="B10" s="3" t="n"/>
+      <c r="C10" s="3" t="n"/>
+      <c r="D10" s="3" t="n"/>
+      <c r="E10" s="3" t="n"/>
+      <c r="F10" s="3" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="4" t="n"/>
+      <c r="J10" s="4" t="n"/>
+      <c r="K10" s="4" t="n"/>
+      <c r="L10" s="4" t="n"/>
+      <c r="M10" s="4" t="n"/>
+      <c r="N10" s="4" t="n"/>
+      <c r="O10" s="4" t="n"/>
+      <c r="P10" s="4" t="n"/>
+      <c r="S10" s="57" t="n"/>
+      <c r="T10" s="56" t="n"/>
+      <c r="Z10" s="57" t="n"/>
     </row>
     <row r="11" ht="15.6" customHeight="1" s="42">
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+      <c r="M11" s="6" t="n"/>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+      <c r="Q11" s="6" t="n"/>
+      <c r="R11" s="6" t="n"/>
+      <c r="S11" s="6" t="n"/>
+      <c r="T11" s="6" t="n"/>
+      <c r="U11" s="6" t="n"/>
+      <c r="V11" s="6" t="n"/>
+      <c r="W11" s="6" t="n"/>
+      <c r="X11" s="6" t="n"/>
+      <c r="Y11" s="6" t="n"/>
+      <c r="Z11" s="6" t="n"/>
+      <c r="AA11" s="6" t="n"/>
+      <c r="AB11" s="6" t="n"/>
+      <c r="AC11" s="6" t="n"/>
+      <c r="AD11" s="6" t="n"/>
+      <c r="AE11" s="6" t="n"/>
+      <c r="AF11" s="6" t="n"/>
+      <c r="AG11" s="6" t="n"/>
+      <c r="AH11" s="6" t="n"/>
+      <c r="AI11" s="6" t="n"/>
+      <c r="AJ11" s="6" t="n"/>
+      <c r="AK11" s="6" t="n"/>
+      <c r="AL11" s="6" t="n"/>
+      <c r="AM11" s="6" t="n"/>
+      <c r="AN11" s="6" t="n"/>
+      <c r="AO11" s="6" t="n"/>
+      <c r="AP11" s="6" t="n"/>
+      <c r="AQ11" s="6" t="n"/>
+      <c r="AR11" s="6" t="n"/>
+      <c r="AS11" s="6" t="n"/>
+      <c r="AT11" s="6" t="n"/>
+      <c r="AU11" s="6" t="n"/>
+      <c r="AV11" s="6" t="n"/>
+      <c r="AW11" s="6" t="n"/>
+      <c r="AX11" s="6" t="n"/>
+      <c r="AY11" s="6" t="n"/>
+      <c r="AZ11" s="6" t="n"/>
+      <c r="BA11" s="6" t="n"/>
+      <c r="BB11" s="6" t="n"/>
+      <c r="BC11" s="6" t="n"/>
+      <c r="BD11" s="6" t="n"/>
+      <c r="BE11" s="6" t="n"/>
+      <c r="BF11" s="6" t="n"/>
+      <c r="BG11" s="6" t="n"/>
+      <c r="BH11" s="6" t="n"/>
+      <c r="BI11" s="6" t="n"/>
+      <c r="BJ11" s="6" t="n"/>
+      <c r="BK11" s="6" t="n"/>
+      <c r="BL11" s="6" t="n"/>
+      <c r="BM11" s="6" t="n"/>
+      <c r="BN11" s="6" t="n"/>
+      <c r="BO11" s="6" t="n"/>
+      <c r="BP11" s="7" t="n"/>
+    </row>
+    <row r="12" ht="19.95" customHeight="1" s="42">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>GRUP FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="C11" s="33" t="n"/>
-      <c r="D11" s="33" t="n"/>
-      <c r="E11" s="33" t="n"/>
-      <c r="F11" s="33" t="n"/>
-      <c r="G11" s="33" t="n"/>
-      <c r="H11" s="33" t="n"/>
-      <c r="I11" s="33" t="n"/>
-      <c r="J11" s="33" t="n"/>
-      <c r="K11" s="33" t="n"/>
-      <c r="L11" s="33" t="n"/>
-      <c r="M11" s="33" t="n"/>
-      <c r="N11" s="33" t="n"/>
-      <c r="O11" s="33" t="n"/>
-      <c r="P11" s="33" t="n"/>
-      <c r="Q11" s="33" t="n"/>
-      <c r="R11" s="33" t="n"/>
-      <c r="S11" s="33" t="n"/>
-      <c r="T11" s="33" t="n"/>
-      <c r="U11" s="33" t="n"/>
-      <c r="V11" s="33" t="n"/>
-      <c r="W11" s="33" t="n"/>
-      <c r="X11" s="33" t="n"/>
-      <c r="Y11" s="33" t="n"/>
-      <c r="Z11" s="33" t="n"/>
-      <c r="AA11" s="34" t="inlineStr">
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="33" t="n"/>
+      <c r="F12" s="33" t="n"/>
+      <c r="G12" s="33" t="n"/>
+      <c r="H12" s="33" t="n"/>
+      <c r="I12" s="33" t="n"/>
+      <c r="J12" s="33" t="n"/>
+      <c r="K12" s="33" t="n"/>
+      <c r="L12" s="33" t="n"/>
+      <c r="M12" s="33" t="n"/>
+      <c r="N12" s="33" t="n"/>
+      <c r="O12" s="33" t="n"/>
+      <c r="P12" s="33" t="n"/>
+      <c r="Q12" s="33" t="n"/>
+      <c r="R12" s="33" t="n"/>
+      <c r="S12" s="33" t="n"/>
+      <c r="T12" s="33" t="n"/>
+      <c r="U12" s="33" t="n"/>
+      <c r="V12" s="33" t="n"/>
+      <c r="W12" s="33" t="n"/>
+      <c r="X12" s="33" t="n"/>
+      <c r="Y12" s="33" t="n"/>
+      <c r="Z12" s="33" t="n"/>
+      <c r="AA12" s="34" t="inlineStr">
         <is>
           <t>FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="AB11" s="33" t="n"/>
-      <c r="AC11" s="33" t="n"/>
-      <c r="AD11" s="33" t="n"/>
-      <c r="AE11" s="33" t="n"/>
-      <c r="AF11" s="33" t="n"/>
-      <c r="AG11" s="33" t="n"/>
-      <c r="AH11" s="33" t="n"/>
-      <c r="AI11" s="33" t="n"/>
-      <c r="AJ11" s="33" t="n"/>
-      <c r="AK11" s="33" t="n"/>
-      <c r="AL11" s="33" t="n"/>
-      <c r="AM11" s="33" t="n"/>
-      <c r="AN11" s="33" t="n"/>
-      <c r="AO11" s="33" t="n"/>
-      <c r="AP11" s="34" t="inlineStr">
+      <c r="AB12" s="33" t="n"/>
+      <c r="AC12" s="33" t="n"/>
+      <c r="AD12" s="33" t="n"/>
+      <c r="AE12" s="33" t="n"/>
+      <c r="AF12" s="33" t="n"/>
+      <c r="AG12" s="33" t="n"/>
+      <c r="AH12" s="33" t="n"/>
+      <c r="AI12" s="33" t="n"/>
+      <c r="AJ12" s="33" t="n"/>
+      <c r="AK12" s="33" t="n"/>
+      <c r="AL12" s="33" t="n"/>
+      <c r="AM12" s="33" t="n"/>
+      <c r="AN12" s="33" t="n"/>
+      <c r="AO12" s="33" t="n"/>
+      <c r="AP12" s="34" t="inlineStr">
         <is>
           <t>FREKANS SAPMALARI</t>
         </is>
       </c>
-      <c r="AQ11" s="33" t="n"/>
-      <c r="AR11" s="33" t="n"/>
-      <c r="AS11" s="33" t="n"/>
-      <c r="AT11" s="33" t="n"/>
-      <c r="AU11" s="33" t="n"/>
-      <c r="AV11" s="33" t="n"/>
-      <c r="AW11" s="33" t="n"/>
-      <c r="AX11" s="33" t="n"/>
-      <c r="AY11" s="33" t="n"/>
-      <c r="AZ11" s="33" t="n"/>
-      <c r="BA11" s="33" t="n"/>
-      <c r="BB11" s="33" t="n"/>
-      <c r="BC11" s="33" t="n"/>
-      <c r="BD11" s="34" t="inlineStr">
+      <c r="AQ12" s="33" t="n"/>
+      <c r="AR12" s="33" t="n"/>
+      <c r="AS12" s="33" t="n"/>
+      <c r="AT12" s="33" t="n"/>
+      <c r="AU12" s="33" t="n"/>
+      <c r="AV12" s="33" t="n"/>
+      <c r="AW12" s="33" t="n"/>
+      <c r="AX12" s="33" t="n"/>
+      <c r="AY12" s="33" t="n"/>
+      <c r="AZ12" s="33" t="n"/>
+      <c r="BA12" s="33" t="n"/>
+      <c r="BB12" s="33" t="n"/>
+      <c r="BC12" s="33" t="n"/>
+      <c r="BD12" s="34" t="inlineStr">
         <is>
           <t>KAYIP FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="BE11" s="33" t="n"/>
-      <c r="BF11" s="33" t="n"/>
-      <c r="BG11" s="33" t="n"/>
-      <c r="BH11" s="33" t="n"/>
-      <c r="BI11" s="33" t="n"/>
-      <c r="BJ11" s="33" t="n"/>
-      <c r="BK11" s="33" t="n"/>
-      <c r="BL11" s="33" t="n"/>
-      <c r="BM11" s="33" t="n"/>
-      <c r="BN11" s="33" t="n"/>
-      <c r="BO11" s="33" t="n"/>
-      <c r="BP11" s="15" t="n"/>
-    </row>
-    <row r="12" ht="19.95" customHeight="1" s="42">
-      <c r="B12" s="84" t="inlineStr">
+      <c r="BE12" s="33" t="n"/>
+      <c r="BF12" s="33" t="n"/>
+      <c r="BG12" s="33" t="n"/>
+      <c r="BH12" s="33" t="n"/>
+      <c r="BI12" s="33" t="n"/>
+      <c r="BJ12" s="33" t="n"/>
+      <c r="BK12" s="33" t="n"/>
+      <c r="BL12" s="33" t="n"/>
+      <c r="BM12" s="33" t="n"/>
+      <c r="BN12" s="33" t="n"/>
+      <c r="BO12" s="33" t="n"/>
+      <c r="BP12" s="15" t="n"/>
+    </row>
+    <row r="13" ht="19.95" customHeight="1" s="42">
+      <c r="B13" s="84" t="inlineStr">
         <is>
           <t>GRUP TANIMI</t>
         </is>
       </c>
-      <c r="C12" s="175" t="n"/>
-      <c r="D12" s="176" t="n"/>
-      <c r="E12" s="85" t="inlineStr">
+      <c r="C13" s="175" t="n"/>
+      <c r="D13" s="176" t="n"/>
+      <c r="E13" s="85" t="inlineStr">
         <is>
           <t>HEDEF FREKANS SAYISI</t>
         </is>
       </c>
-      <c r="F12" s="175" t="n"/>
-      <c r="G12" s="176" t="n"/>
-      <c r="H12" s="85" t="inlineStr">
+      <c r="F13" s="175" t="n"/>
+      <c r="G13" s="176" t="n"/>
+      <c r="H13" s="85" t="inlineStr">
         <is>
           <t>TAMAMLANMIŞ FREKANS SAYISI</t>
         </is>
       </c>
-      <c r="I12" s="175" t="n"/>
-      <c r="J12" s="176" t="n"/>
-      <c r="K12" s="85" t="inlineStr">
+      <c r="I13" s="175" t="n"/>
+      <c r="J13" s="176" t="n"/>
+      <c r="K13" s="85" t="inlineStr">
         <is>
           <t>ZAMANINDA GERÇEKLEŞEN İŞLEM ORANI</t>
         </is>
       </c>
-      <c r="L12" s="175" t="n"/>
-      <c r="M12" s="175" t="n"/>
-      <c r="N12" s="176" t="n"/>
-      <c r="O12" s="85" t="inlineStr">
+      <c r="L13" s="175" t="n"/>
+      <c r="M13" s="175" t="n"/>
+      <c r="N13" s="176" t="n"/>
+      <c r="O13" s="85" t="inlineStr">
         <is>
           <t>SAPMA FREKANS SAYISI</t>
         </is>
       </c>
-      <c r="P12" s="175" t="n"/>
-      <c r="Q12" s="176" t="n"/>
-      <c r="R12" s="85" t="inlineStr">
+      <c r="P13" s="175" t="n"/>
+      <c r="Q13" s="176" t="n"/>
+      <c r="R13" s="85" t="inlineStr">
         <is>
           <t>KAYIP FREKANS SAYISI</t>
         </is>
       </c>
-      <c r="S12" s="175" t="n"/>
-      <c r="T12" s="175" t="n"/>
-      <c r="U12" s="176" t="n"/>
-      <c r="V12" s="177" t="inlineStr">
+      <c r="S13" s="175" t="n"/>
+      <c r="T13" s="175" t="n"/>
+      <c r="U13" s="176" t="n"/>
+      <c r="V13" s="177" t="inlineStr">
         <is>
           <t>GENEL ORAN</t>
         </is>
       </c>
-      <c r="W12" s="175" t="n"/>
-      <c r="X12" s="176" t="n"/>
-      <c r="AA12" s="53" t="inlineStr">
+      <c r="W13" s="175" t="n"/>
+      <c r="X13" s="176" t="n"/>
+      <c r="AA13" s="53" t="inlineStr">
         <is>
           <t>Toplam Frekans Sayısı</t>
-        </is>
-      </c>
-      <c r="AB12" s="158" t="n"/>
-      <c r="AC12" s="158" t="n"/>
-      <c r="AD12" s="158" t="n"/>
-      <c r="AE12" s="158" t="n"/>
-      <c r="AF12" s="158" t="n"/>
-      <c r="AG12" s="158" t="n"/>
-      <c r="AH12" s="158" t="n"/>
-      <c r="AI12" s="158" t="n"/>
-      <c r="AJ12" s="159" t="n"/>
-      <c r="AK12" s="54" t="n"/>
-      <c r="AL12" s="158" t="n"/>
-      <c r="AM12" s="158" t="n"/>
-      <c r="AN12" s="159" t="n"/>
-      <c r="AP12" s="53" t="inlineStr">
-        <is>
-          <t>Toplam Frekans Sayısı</t>
-        </is>
-      </c>
-      <c r="AQ12" s="158" t="n"/>
-      <c r="AR12" s="158" t="n"/>
-      <c r="AS12" s="158" t="n"/>
-      <c r="AT12" s="158" t="n"/>
-      <c r="AU12" s="158" t="n"/>
-      <c r="AV12" s="158" t="n"/>
-      <c r="AW12" s="158" t="n"/>
-      <c r="AX12" s="158" t="n"/>
-      <c r="AY12" s="159" t="n"/>
-      <c r="AZ12" s="54" t="n"/>
-      <c r="BA12" s="158" t="n"/>
-      <c r="BB12" s="159" t="n"/>
-      <c r="BC12" s="16" t="n"/>
-      <c r="BD12" s="53" t="inlineStr">
-        <is>
-          <t>Toplam Frekans Sayısı</t>
-        </is>
-      </c>
-      <c r="BE12" s="158" t="n"/>
-      <c r="BF12" s="158" t="n"/>
-      <c r="BG12" s="158" t="n"/>
-      <c r="BH12" s="158" t="n"/>
-      <c r="BI12" s="158" t="n"/>
-      <c r="BJ12" s="158" t="n"/>
-      <c r="BK12" s="158" t="n"/>
-      <c r="BL12" s="158" t="n"/>
-      <c r="BM12" s="159" t="n"/>
-      <c r="BN12" s="54" t="n"/>
-      <c r="BO12" s="159" t="n"/>
-      <c r="BP12" s="8" t="n"/>
-      <c r="BR12" t="inlineStr">
-        <is>
-          <t>"</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="19.95" customHeight="1" s="42">
-      <c r="B13" s="178" t="n"/>
-      <c r="C13" s="179" t="n"/>
-      <c r="D13" s="180" t="n"/>
-      <c r="E13" s="181" t="n"/>
-      <c r="F13" s="179" t="n"/>
-      <c r="G13" s="180" t="n"/>
-      <c r="H13" s="181" t="n"/>
-      <c r="I13" s="179" t="n"/>
-      <c r="J13" s="180" t="n"/>
-      <c r="K13" s="181" t="n"/>
-      <c r="L13" s="179" t="n"/>
-      <c r="M13" s="179" t="n"/>
-      <c r="N13" s="180" t="n"/>
-      <c r="O13" s="181" t="n"/>
-      <c r="P13" s="179" t="n"/>
-      <c r="Q13" s="180" t="n"/>
-      <c r="R13" s="181" t="n"/>
-      <c r="S13" s="179" t="n"/>
-      <c r="T13" s="179" t="n"/>
-      <c r="U13" s="180" t="n"/>
-      <c r="V13" s="179" t="n"/>
-      <c r="W13" s="179" t="n"/>
-      <c r="X13" s="180" t="n"/>
-      <c r="AA13" s="53" t="inlineStr">
-        <is>
-          <t>Tamamlanmış Frekans Sayısı</t>
         </is>
       </c>
       <c r="AB13" s="158" t="n"/>
@@ -4053,13 +3996,13 @@
       <c r="AH13" s="158" t="n"/>
       <c r="AI13" s="158" t="n"/>
       <c r="AJ13" s="159" t="n"/>
-      <c r="AK13" s="60" t="n"/>
+      <c r="AK13" s="54" t="n"/>
       <c r="AL13" s="158" t="n"/>
       <c r="AM13" s="158" t="n"/>
       <c r="AN13" s="159" t="n"/>
       <c r="AP13" s="53" t="inlineStr">
         <is>
-          <t>Sapma Frekans Sayısı</t>
+          <t>Toplam Frekans Sayısı</t>
         </is>
       </c>
       <c r="AQ13" s="158" t="n"/>
@@ -4077,7 +4020,7 @@
       <c r="BC13" s="16" t="n"/>
       <c r="BD13" s="53" t="inlineStr">
         <is>
-          <t>Kayıp Frekans Sayısı</t>
+          <t>Toplam Frekans Sayısı</t>
         </is>
       </c>
       <c r="BE13" s="158" t="n"/>
@@ -4092,37 +4035,39 @@
       <c r="BN13" s="54" t="n"/>
       <c r="BO13" s="159" t="n"/>
       <c r="BP13" s="8" t="n"/>
-      <c r="BQ13" s="13" t="n">
-        <v>0.3</v>
+      <c r="BR13" t="inlineStr">
+        <is>
+          <t>"</t>
+        </is>
       </c>
     </row>
     <row r="14" ht="22.2" customHeight="1" s="42">
-      <c r="B14" s="90" t="n"/>
-      <c r="C14" s="158" t="n"/>
-      <c r="D14" s="159" t="n"/>
-      <c r="E14" s="59" t="n"/>
-      <c r="F14" s="158" t="n"/>
-      <c r="G14" s="159" t="n"/>
-      <c r="H14" s="58" t="n"/>
-      <c r="I14" s="158" t="n"/>
-      <c r="J14" s="159" t="n"/>
-      <c r="K14" s="86" t="n"/>
-      <c r="L14" s="158" t="n"/>
-      <c r="M14" s="158" t="n"/>
-      <c r="N14" s="159" t="n"/>
-      <c r="O14" s="58" t="n"/>
-      <c r="P14" s="158" t="n"/>
-      <c r="Q14" s="159" t="n"/>
-      <c r="R14" s="58" t="n"/>
-      <c r="S14" s="158" t="n"/>
-      <c r="T14" s="158" t="n"/>
-      <c r="U14" s="159" t="n"/>
-      <c r="V14" s="182" t="n"/>
-      <c r="W14" s="158" t="n"/>
-      <c r="X14" s="159" t="n"/>
+      <c r="B14" s="178" t="n"/>
+      <c r="C14" s="179" t="n"/>
+      <c r="D14" s="180" t="n"/>
+      <c r="E14" s="181" t="n"/>
+      <c r="F14" s="179" t="n"/>
+      <c r="G14" s="180" t="n"/>
+      <c r="H14" s="181" t="n"/>
+      <c r="I14" s="179" t="n"/>
+      <c r="J14" s="180" t="n"/>
+      <c r="K14" s="181" t="n"/>
+      <c r="L14" s="179" t="n"/>
+      <c r="M14" s="179" t="n"/>
+      <c r="N14" s="180" t="n"/>
+      <c r="O14" s="181" t="n"/>
+      <c r="P14" s="179" t="n"/>
+      <c r="Q14" s="180" t="n"/>
+      <c r="R14" s="181" t="n"/>
+      <c r="S14" s="179" t="n"/>
+      <c r="T14" s="179" t="n"/>
+      <c r="U14" s="180" t="n"/>
+      <c r="V14" s="179" t="n"/>
+      <c r="W14" s="179" t="n"/>
+      <c r="X14" s="180" t="n"/>
       <c r="AA14" s="53" t="inlineStr">
         <is>
-          <t>Gerçekleşen Frekans Sayısı</t>
+          <t>Tamamlanmış Frekans Sayısı</t>
         </is>
       </c>
       <c r="AB14" s="158" t="n"/>
@@ -4140,7 +4085,7 @@
       <c r="AN14" s="159" t="n"/>
       <c r="AP14" s="53" t="inlineStr">
         <is>
-          <t>Sapma Frekans Oranı</t>
+          <t>Sapma Frekans Sayısı</t>
         </is>
       </c>
       <c r="AQ14" s="158" t="n"/>
@@ -4152,13 +4097,13 @@
       <c r="AW14" s="158" t="n"/>
       <c r="AX14" s="158" t="n"/>
       <c r="AY14" s="159" t="n"/>
-      <c r="AZ14" s="55" t="n"/>
+      <c r="AZ14" s="54" t="n"/>
       <c r="BA14" s="158" t="n"/>
       <c r="BB14" s="159" t="n"/>
       <c r="BC14" s="16" t="n"/>
       <c r="BD14" s="53" t="inlineStr">
         <is>
-          <t>Kayıp Frekans Oranı</t>
+          <t>Kayıp Frekans Sayısı</t>
         </is>
       </c>
       <c r="BE14" s="158" t="n"/>
@@ -4170,11 +4115,11 @@
       <c r="BK14" s="158" t="n"/>
       <c r="BL14" s="158" t="n"/>
       <c r="BM14" s="159" t="n"/>
-      <c r="BN14" s="55" t="n"/>
+      <c r="BN14" s="54" t="n"/>
       <c r="BO14" s="159" t="n"/>
       <c r="BP14" s="8" t="n"/>
-      <c r="BQ14" t="n">
-        <v>0.2</v>
+      <c r="BQ14" s="13" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="15" ht="22.2" customHeight="1" s="42">
@@ -4184,7 +4129,7 @@
       <c r="E15" s="59" t="n"/>
       <c r="F15" s="158" t="n"/>
       <c r="G15" s="159" t="n"/>
-      <c r="H15" s="59" t="n"/>
+      <c r="H15" s="58" t="n"/>
       <c r="I15" s="158" t="n"/>
       <c r="J15" s="159" t="n"/>
       <c r="K15" s="86" t="n"/>
@@ -4203,7 +4148,7 @@
       <c r="X15" s="159" t="n"/>
       <c r="AA15" s="53" t="inlineStr">
         <is>
-          <t>Sapma Frekans Sayısı</t>
+          <t>Gerçekleşen Frekans Sayısı</t>
         </is>
       </c>
       <c r="AB15" s="158" t="n"/>
@@ -4215,11 +4160,48 @@
       <c r="AH15" s="158" t="n"/>
       <c r="AI15" s="158" t="n"/>
       <c r="AJ15" s="159" t="n"/>
-      <c r="AK15" s="54" t="n"/>
+      <c r="AK15" s="60" t="n"/>
       <c r="AL15" s="158" t="n"/>
       <c r="AM15" s="158" t="n"/>
       <c r="AN15" s="159" t="n"/>
+      <c r="AP15" s="53" t="inlineStr">
+        <is>
+          <t>Sapma Frekans Oranı</t>
+        </is>
+      </c>
+      <c r="AQ15" s="158" t="n"/>
+      <c r="AR15" s="158" t="n"/>
+      <c r="AS15" s="158" t="n"/>
+      <c r="AT15" s="158" t="n"/>
+      <c r="AU15" s="158" t="n"/>
+      <c r="AV15" s="158" t="n"/>
+      <c r="AW15" s="158" t="n"/>
+      <c r="AX15" s="158" t="n"/>
+      <c r="AY15" s="159" t="n"/>
+      <c r="AZ15" s="55" t="n"/>
+      <c r="BA15" s="158" t="n"/>
+      <c r="BB15" s="159" t="n"/>
+      <c r="BC15" s="16" t="n"/>
+      <c r="BD15" s="53" t="inlineStr">
+        <is>
+          <t>Kayıp Frekans Oranı</t>
+        </is>
+      </c>
+      <c r="BE15" s="158" t="n"/>
+      <c r="BF15" s="158" t="n"/>
+      <c r="BG15" s="158" t="n"/>
+      <c r="BH15" s="158" t="n"/>
+      <c r="BI15" s="158" t="n"/>
+      <c r="BJ15" s="158" t="n"/>
+      <c r="BK15" s="158" t="n"/>
+      <c r="BL15" s="158" t="n"/>
+      <c r="BM15" s="159" t="n"/>
+      <c r="BN15" s="55" t="n"/>
+      <c r="BO15" s="159" t="n"/>
       <c r="BP15" s="8" t="n"/>
+      <c r="BQ15" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="16" ht="22.2" customHeight="1" s="42">
       <c r="B16" s="90" t="n"/>
@@ -4247,7 +4229,7 @@
       <c r="X16" s="159" t="n"/>
       <c r="AA16" s="53" t="inlineStr">
         <is>
-          <t>Kayıp Frekans Sayısı</t>
+          <t>Sapma Frekans Sayısı</t>
         </is>
       </c>
       <c r="AB16" s="158" t="n"/>
@@ -4272,7 +4254,7 @@
       <c r="E17" s="59" t="n"/>
       <c r="F17" s="158" t="n"/>
       <c r="G17" s="159" t="n"/>
-      <c r="H17" s="58" t="n"/>
+      <c r="H17" s="59" t="n"/>
       <c r="I17" s="158" t="n"/>
       <c r="J17" s="159" t="n"/>
       <c r="K17" s="86" t="n"/>
@@ -4291,7 +4273,7 @@
       <c r="X17" s="159" t="n"/>
       <c r="AA17" s="53" t="inlineStr">
         <is>
-          <t>Başarı Ortalaması</t>
+          <t>Kayıp Frekans Sayısı</t>
         </is>
       </c>
       <c r="AB17" s="158" t="n"/>
@@ -4303,7 +4285,7 @@
       <c r="AH17" s="158" t="n"/>
       <c r="AI17" s="158" t="n"/>
       <c r="AJ17" s="159" t="n"/>
-      <c r="AK17" s="55" t="n"/>
+      <c r="AK17" s="54" t="n"/>
       <c r="AL17" s="158" t="n"/>
       <c r="AM17" s="158" t="n"/>
       <c r="AN17" s="159" t="n"/>
@@ -4333,10 +4315,50 @@
       <c r="V18" s="182" t="n"/>
       <c r="W18" s="158" t="n"/>
       <c r="X18" s="159" t="n"/>
+      <c r="AA18" s="53" t="inlineStr">
+        <is>
+          <t>Başarı Ortalaması</t>
+        </is>
+      </c>
+      <c r="AB18" s="158" t="n"/>
+      <c r="AC18" s="158" t="n"/>
+      <c r="AD18" s="158" t="n"/>
+      <c r="AE18" s="158" t="n"/>
+      <c r="AF18" s="158" t="n"/>
+      <c r="AG18" s="158" t="n"/>
+      <c r="AH18" s="158" t="n"/>
+      <c r="AI18" s="158" t="n"/>
+      <c r="AJ18" s="159" t="n"/>
+      <c r="AK18" s="55" t="n"/>
+      <c r="AL18" s="158" t="n"/>
+      <c r="AM18" s="158" t="n"/>
+      <c r="AN18" s="159" t="n"/>
       <c r="BP18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="B19" s="9" t="n"/>
+      <c r="B19" s="90" t="n"/>
+      <c r="C19" s="158" t="n"/>
+      <c r="D19" s="159" t="n"/>
+      <c r="E19" s="59" t="n"/>
+      <c r="F19" s="158" t="n"/>
+      <c r="G19" s="159" t="n"/>
+      <c r="H19" s="58" t="n"/>
+      <c r="I19" s="158" t="n"/>
+      <c r="J19" s="159" t="n"/>
+      <c r="K19" s="86" t="n"/>
+      <c r="L19" s="158" t="n"/>
+      <c r="M19" s="158" t="n"/>
+      <c r="N19" s="159" t="n"/>
+      <c r="O19" s="58" t="n"/>
+      <c r="P19" s="158" t="n"/>
+      <c r="Q19" s="159" t="n"/>
+      <c r="R19" s="58" t="n"/>
+      <c r="S19" s="158" t="n"/>
+      <c r="T19" s="158" t="n"/>
+      <c r="U19" s="159" t="n"/>
+      <c r="V19" s="182" t="n"/>
+      <c r="W19" s="158" t="n"/>
+      <c r="X19" s="159" t="n"/>
       <c r="BP19" s="8" t="n"/>
     </row>
     <row r="20">
@@ -4376,142 +4398,146 @@
       <c r="BP28" s="8" t="n"/>
     </row>
     <row r="29" ht="22.8" customHeight="1" s="42" thickBot="1">
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="11" t="n"/>
-      <c r="I29" s="11" t="n"/>
-      <c r="J29" s="11" t="n"/>
-      <c r="K29" s="11" t="n"/>
-      <c r="L29" s="11" t="n"/>
-      <c r="M29" s="11" t="n"/>
-      <c r="N29" s="11" t="n"/>
-      <c r="O29" s="11" t="n"/>
-      <c r="P29" s="11" t="n"/>
-      <c r="Q29" s="11" t="n"/>
-      <c r="R29" s="11" t="n"/>
-      <c r="S29" s="11" t="n"/>
-      <c r="T29" s="11" t="n"/>
-      <c r="U29" s="11" t="n"/>
-      <c r="V29" s="11" t="n"/>
-      <c r="W29" s="11" t="n"/>
-      <c r="X29" s="11" t="n"/>
-      <c r="Y29" s="11" t="n"/>
-      <c r="Z29" s="11" t="n"/>
-      <c r="AA29" s="11" t="n"/>
-      <c r="AB29" s="11" t="n"/>
-      <c r="AC29" s="11" t="n"/>
-      <c r="AD29" s="11" t="n"/>
-      <c r="AE29" s="11" t="n"/>
-      <c r="AF29" s="11" t="n"/>
-      <c r="AG29" s="11" t="n"/>
-      <c r="AH29" s="11" t="n"/>
-      <c r="AI29" s="11" t="n"/>
-      <c r="AJ29" s="11" t="n"/>
-      <c r="AK29" s="11" t="n"/>
-      <c r="AL29" s="11" t="n"/>
-      <c r="AM29" s="11" t="n"/>
-      <c r="AN29" s="11" t="n"/>
-      <c r="AO29" s="11" t="n"/>
-      <c r="AP29" s="11" t="n"/>
-      <c r="AQ29" s="11" t="n"/>
-      <c r="AR29" s="11" t="n"/>
-      <c r="AS29" s="11" t="n"/>
-      <c r="AT29" s="11" t="n"/>
-      <c r="AU29" s="11" t="n"/>
-      <c r="AV29" s="11" t="n"/>
-      <c r="AW29" s="11" t="n"/>
-      <c r="AX29" s="11" t="n"/>
-      <c r="AY29" s="11" t="n"/>
-      <c r="AZ29" s="11" t="n"/>
-      <c r="BA29" s="11" t="n"/>
-      <c r="BB29" s="11" t="n"/>
-      <c r="BC29" s="11" t="n"/>
-      <c r="BD29" s="11" t="n"/>
-      <c r="BE29" s="11" t="n"/>
-      <c r="BF29" s="11" t="n"/>
-      <c r="BG29" s="11" t="n"/>
-      <c r="BH29" s="11" t="n"/>
-      <c r="BI29" s="11" t="n"/>
-      <c r="BJ29" s="11" t="n"/>
-      <c r="BK29" s="11" t="n"/>
-      <c r="BL29" s="11" t="n"/>
-      <c r="BM29" s="11" t="n"/>
-      <c r="BN29" s="11" t="n"/>
-      <c r="BO29" s="11" t="n"/>
-      <c r="BP29" s="12" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="BP29" s="8" t="n"/>
     </row>
     <row r="30" ht="31.95" customHeight="1" s="42">
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="6" t="n"/>
-      <c r="J30" s="6" t="n"/>
-      <c r="K30" s="6" t="n"/>
-      <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6" t="n"/>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="6" t="n"/>
-      <c r="P30" s="6" t="n"/>
-      <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="6" t="n"/>
-      <c r="S30" s="6" t="n"/>
-      <c r="T30" s="6" t="n"/>
-      <c r="U30" s="6" t="n"/>
-      <c r="V30" s="6" t="n"/>
-      <c r="W30" s="6" t="n"/>
-      <c r="X30" s="6" t="n"/>
-      <c r="Y30" s="6" t="n"/>
-      <c r="Z30" s="6" t="n"/>
-      <c r="AA30" s="6" t="n"/>
-      <c r="AB30" s="6" t="n"/>
-      <c r="AC30" s="6" t="n"/>
-      <c r="AD30" s="6" t="n"/>
-      <c r="AE30" s="6" t="n"/>
-      <c r="AF30" s="6" t="n"/>
-      <c r="AG30" s="6" t="n"/>
-      <c r="AH30" s="6" t="n"/>
-      <c r="AI30" s="6" t="n"/>
-      <c r="AJ30" s="6" t="n"/>
-      <c r="AK30" s="6" t="n"/>
-      <c r="AL30" s="6" t="n"/>
-      <c r="AM30" s="6" t="n"/>
-      <c r="AN30" s="6" t="n"/>
-      <c r="AO30" s="6" t="n"/>
-      <c r="AP30" s="6" t="n"/>
-      <c r="AQ30" s="6" t="n"/>
-      <c r="AR30" s="6" t="n"/>
-      <c r="AS30" s="6" t="n"/>
-      <c r="AT30" s="6" t="n"/>
-      <c r="AU30" s="6" t="n"/>
-      <c r="AV30" s="6" t="n"/>
-      <c r="AW30" s="6" t="n"/>
-      <c r="AX30" s="6" t="n"/>
-      <c r="AY30" s="6" t="n"/>
-      <c r="AZ30" s="6" t="n"/>
-      <c r="BA30" s="6" t="n"/>
-      <c r="BB30" s="6" t="n"/>
-      <c r="BC30" s="6" t="n"/>
-      <c r="BD30" s="6" t="n"/>
-      <c r="BE30" s="6" t="n"/>
-      <c r="BF30" s="6" t="n"/>
-      <c r="BG30" s="6" t="n"/>
-      <c r="BH30" s="6" t="n"/>
-      <c r="BI30" s="6" t="n"/>
-      <c r="BJ30" s="6" t="n"/>
-      <c r="BK30" s="6" t="n"/>
-      <c r="BL30" s="6" t="n"/>
-      <c r="BM30" s="6" t="n"/>
-      <c r="BN30" s="6" t="n"/>
-      <c r="BO30" s="6" t="n"/>
-      <c r="BP30" s="6" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="11" t="n"/>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="11" t="n"/>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="11" t="n"/>
+      <c r="I30" s="11" t="n"/>
+      <c r="J30" s="11" t="n"/>
+      <c r="K30" s="11" t="n"/>
+      <c r="L30" s="11" t="n"/>
+      <c r="M30" s="11" t="n"/>
+      <c r="N30" s="11" t="n"/>
+      <c r="O30" s="11" t="n"/>
+      <c r="P30" s="11" t="n"/>
+      <c r="Q30" s="11" t="n"/>
+      <c r="R30" s="11" t="n"/>
+      <c r="S30" s="11" t="n"/>
+      <c r="T30" s="11" t="n"/>
+      <c r="U30" s="11" t="n"/>
+      <c r="V30" s="11" t="n"/>
+      <c r="W30" s="11" t="n"/>
+      <c r="X30" s="11" t="n"/>
+      <c r="Y30" s="11" t="n"/>
+      <c r="Z30" s="11" t="n"/>
+      <c r="AA30" s="11" t="n"/>
+      <c r="AB30" s="11" t="n"/>
+      <c r="AC30" s="11" t="n"/>
+      <c r="AD30" s="11" t="n"/>
+      <c r="AE30" s="11" t="n"/>
+      <c r="AF30" s="11" t="n"/>
+      <c r="AG30" s="11" t="n"/>
+      <c r="AH30" s="11" t="n"/>
+      <c r="AI30" s="11" t="n"/>
+      <c r="AJ30" s="11" t="n"/>
+      <c r="AK30" s="11" t="n"/>
+      <c r="AL30" s="11" t="n"/>
+      <c r="AM30" s="11" t="n"/>
+      <c r="AN30" s="11" t="n"/>
+      <c r="AO30" s="11" t="n"/>
+      <c r="AP30" s="11" t="n"/>
+      <c r="AQ30" s="11" t="n"/>
+      <c r="AR30" s="11" t="n"/>
+      <c r="AS30" s="11" t="n"/>
+      <c r="AT30" s="11" t="n"/>
+      <c r="AU30" s="11" t="n"/>
+      <c r="AV30" s="11" t="n"/>
+      <c r="AW30" s="11" t="n"/>
+      <c r="AX30" s="11" t="n"/>
+      <c r="AY30" s="11" t="n"/>
+      <c r="AZ30" s="11" t="n"/>
+      <c r="BA30" s="11" t="n"/>
+      <c r="BB30" s="11" t="n"/>
+      <c r="BC30" s="11" t="n"/>
+      <c r="BD30" s="11" t="n"/>
+      <c r="BE30" s="11" t="n"/>
+      <c r="BF30" s="11" t="n"/>
+      <c r="BG30" s="11" t="n"/>
+      <c r="BH30" s="11" t="n"/>
+      <c r="BI30" s="11" t="n"/>
+      <c r="BJ30" s="11" t="n"/>
+      <c r="BK30" s="11" t="n"/>
+      <c r="BL30" s="11" t="n"/>
+      <c r="BM30" s="11" t="n"/>
+      <c r="BN30" s="11" t="n"/>
+      <c r="BO30" s="11" t="n"/>
+      <c r="BP30" s="12" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+      <c r="M31" s="6" t="n"/>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="6" t="n"/>
+      <c r="P31" s="6" t="n"/>
+      <c r="Q31" s="6" t="n"/>
+      <c r="R31" s="6" t="n"/>
+      <c r="S31" s="6" t="n"/>
+      <c r="T31" s="6" t="n"/>
+      <c r="U31" s="6" t="n"/>
+      <c r="V31" s="6" t="n"/>
+      <c r="W31" s="6" t="n"/>
+      <c r="X31" s="6" t="n"/>
+      <c r="Y31" s="6" t="n"/>
+      <c r="Z31" s="6" t="n"/>
+      <c r="AA31" s="6" t="n"/>
+      <c r="AB31" s="6" t="n"/>
+      <c r="AC31" s="6" t="n"/>
+      <c r="AD31" s="6" t="n"/>
+      <c r="AE31" s="6" t="n"/>
+      <c r="AF31" s="6" t="n"/>
+      <c r="AG31" s="6" t="n"/>
+      <c r="AH31" s="6" t="n"/>
+      <c r="AI31" s="6" t="n"/>
+      <c r="AJ31" s="6" t="n"/>
+      <c r="AK31" s="6" t="n"/>
+      <c r="AL31" s="6" t="n"/>
+      <c r="AM31" s="6" t="n"/>
+      <c r="AN31" s="6" t="n"/>
+      <c r="AO31" s="6" t="n"/>
+      <c r="AP31" s="6" t="n"/>
+      <c r="AQ31" s="6" t="n"/>
+      <c r="AR31" s="6" t="n"/>
+      <c r="AS31" s="6" t="n"/>
+      <c r="AT31" s="6" t="n"/>
+      <c r="AU31" s="6" t="n"/>
+      <c r="AV31" s="6" t="n"/>
+      <c r="AW31" s="6" t="n"/>
+      <c r="AX31" s="6" t="n"/>
+      <c r="AY31" s="6" t="n"/>
+      <c r="AZ31" s="6" t="n"/>
+      <c r="BA31" s="6" t="n"/>
+      <c r="BB31" s="6" t="n"/>
+      <c r="BC31" s="6" t="n"/>
+      <c r="BD31" s="6" t="n"/>
+      <c r="BE31" s="6" t="n"/>
+      <c r="BF31" s="6" t="n"/>
+      <c r="BG31" s="6" t="n"/>
+      <c r="BH31" s="6" t="n"/>
+      <c r="BI31" s="6" t="n"/>
+      <c r="BJ31" s="6" t="n"/>
+      <c r="BK31" s="6" t="n"/>
+      <c r="BL31" s="6" t="n"/>
+      <c r="BM31" s="6" t="n"/>
+      <c r="BN31" s="6" t="n"/>
+      <c r="BO31" s="6" t="n"/>
+      <c r="BP31" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="140">
@@ -4758,7 +4784,7 @@
       <c r="E4" s="36" t="n"/>
       <c r="F4" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="G4" s="59" t="n"/>
@@ -4773,7 +4799,7 @@
       <c r="E5" s="36" t="n"/>
       <c r="F5" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="G5" s="59" t="n"/>
@@ -4788,7 +4814,7 @@
       <c r="E6" s="36" t="n"/>
       <c r="F6" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="G6" s="59" t="n"/>
@@ -4803,7 +4829,7 @@
       <c r="E7" s="36" t="n"/>
       <c r="F7" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="G7" s="59" t="n"/>
@@ -4818,7 +4844,7 @@
       <c r="E8" s="36" t="n"/>
       <c r="F8" s="59" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t> </t>
         </is>
       </c>
       <c r="G8" s="59" t="n"/>
@@ -4926,7 +4952,7 @@
       <c r="F4" s="36" t="n"/>
       <c r="G4" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
     </row>
@@ -4941,7 +4967,7 @@
       <c r="F5" s="36" t="n"/>
       <c r="G5" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
     </row>
@@ -4956,7 +4982,7 @@
       <c r="F6" s="36" t="n"/>
       <c r="G6" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
     </row>
@@ -4971,7 +4997,7 @@
       <c r="F7" s="36" t="n"/>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
     </row>
@@ -4986,7 +5012,7 @@
       <c r="F8" s="36" t="n"/>
       <c r="G8" s="36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  </t>
+          <t>  </t>
         </is>
       </c>
     </row>
@@ -5006,7 +5032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" style="42" min="1" max="1"/>
@@ -5015,6 +5041,7 @@
     <col width="36" customWidth="1" style="42" min="4" max="4"/>
     <col width="22" customWidth="1" style="42" min="5" max="5"/>
     <col width="22" customWidth="1" style="42" min="6" max="6"/>
+    <col width="32" customWidth="1" style="42" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1" s="42">
@@ -5065,6 +5092,11 @@
       <c r="C3" s="184">
         <f>COUNTA(A4:A5000)</f>
         <v/>
+      </c>
+      <c r="G3" s="189" t="inlineStr">
+        <is>
+          <t>KAYIP NEDENİ</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -5135,78 +5167,72 @@
   <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="7.6640625" customWidth="1" style="42" min="1" max="1"/>
-    <col width="13.6640625" customWidth="1" style="25" min="2" max="2"/>
-    <col width="42" bestFit="1" customWidth="1" style="18" min="3" max="3"/>
-    <col width="38" customWidth="1" style="42" min="4" max="4"/>
-    <col width="15.88671875" customWidth="1" style="42" min="5" max="5"/>
-    <col width="16.44140625" customWidth="1" style="42" min="6" max="6"/>
-    <col width="17.33203125" customWidth="1" style="42" min="7" max="7"/>
-    <col width="15.6640625" customWidth="1" style="42" min="8" max="8"/>
-    <col width="22.21875" customWidth="1" style="42" min="9" max="9"/>
-    <col width="26.44140625" customWidth="1" style="42" min="10" max="10"/>
+    <col width="5" customWidth="1" style="42" min="1" max="1"/>
+    <col width="22" customWidth="1" style="25" min="2" max="2"/>
+    <col width="28" bestFit="1" customWidth="1" style="18" min="3" max="3"/>
+    <col width="14" customWidth="1" style="42" min="4" max="4"/>
+    <col width="13" customWidth="1" style="42" min="5" max="5"/>
+    <col width="16" customWidth="1" style="42" min="6" max="6"/>
+    <col width="13" customWidth="1" style="42" min="7" max="7"/>
+    <col width="13" customWidth="1" style="42" min="8" max="8"/>
+    <col width="18" customWidth="1" style="42" min="9" max="9"/>
+    <col width="13" customWidth="1" style="42" min="10" max="10"/>
     <col width="11.44140625" customWidth="1" style="42" min="11" max="11"/>
     <col width="10.88671875" customWidth="1" style="42" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="41.4" customHeight="1" s="42">
-      <c r="A1" s="26" t="inlineStr">
+      <c r="A1" s="189" t="inlineStr">
         <is>
           <t>SN</t>
         </is>
       </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="B1" s="189" t="inlineStr">
         <is>
           <t>GRUP</t>
         </is>
       </c>
-      <c r="C1" s="27" t="inlineStr">
+      <c r="C1" s="189" t="inlineStr">
         <is>
           <t>LOKASYON</t>
         </is>
       </c>
-      <c r="D1" s="28" t="inlineStr">
-        <is>
-          <t>GÖREV TANIMI</t>
-        </is>
-      </c>
-      <c r="E1" s="28" t="inlineStr">
-        <is>
-          <t>GÜNLÜK FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="F1" s="28" t="inlineStr">
-        <is>
-          <t>HEDEF FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="G1" s="28" t="inlineStr">
-        <is>
-          <t>TAMAMLANAN FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="H1" s="28" t="inlineStr">
-        <is>
-          <t>SAPMA FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="I1" s="28" t="inlineStr">
-        <is>
-          <t>KAYIP FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="J1" s="28" t="inlineStr">
-        <is>
-          <t>BAŞARILI İŞLEM ORANI
-Tamamlanan/Hedef</t>
-        </is>
-      </c>
-      <c r="K1" s="28" t="inlineStr">
-        <is>
-          <t>GENEL ORAN
-Tamamlanan+Sapma/Hedef</t>
-        </is>
-      </c>
+      <c r="D1" s="189" t="inlineStr">
+        <is>
+          <t>GÜNLÜK FREKANS</t>
+        </is>
+      </c>
+      <c r="E1" s="189" t="inlineStr">
+        <is>
+          <t>HEDEF FREKANS</t>
+        </is>
+      </c>
+      <c r="F1" s="189" t="inlineStr">
+        <is>
+          <t>TAMAMLANAN FREKANS</t>
+        </is>
+      </c>
+      <c r="G1" s="189" t="inlineStr">
+        <is>
+          <t>SAPMA FREKANS</t>
+        </is>
+      </c>
+      <c r="H1" s="189" t="inlineStr">
+        <is>
+          <t>KAYIP FREKANS</t>
+        </is>
+      </c>
+      <c r="I1" s="189" t="inlineStr">
+        <is>
+          <t>BAŞARILI İŞLEM ORANI</t>
+        </is>
+      </c>
+      <c r="J1" s="189" t="inlineStr">
+        <is>
+          <t>GENEL ORAN</t>
+        </is>
+      </c>
+      <c r="K1" s="28" t="n"/>
     </row>
     <row r="2" ht="21" customHeight="1" s="42">
       <c r="A2" s="185" t="inlineStr">
@@ -5241,10 +5267,7 @@
         <f>IF(F2&gt;0,G2/F2,0)</f>
         <v/>
       </c>
-      <c r="K2" s="186">
-        <f>IF(F2&gt;0,(G2+H2)/F2,0)</f>
-        <v/>
-      </c>
+      <c r="K2" s="186" t="n"/>
     </row>
     <row r="3" ht="15.6" customHeight="1" s="42">
       <c r="A3" s="59" t="n">

</xml_diff>

<commit_message>
excel template: Proje etiketi ve KAYIP NEDENİ konum düzeltildi
- Giriş: Proje etiketi col 1'den col 3'e taşındı (diğer etiketlerle hizalandı)
- Kayıp Frekanslar: KAYIP NEDENİ header G3'ten G2'ye taşındı (header satırı)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/report-templates/QR-SYNC_Genel_Rapor.xlsx
+++ b/public/report-templates/QR-SYNC_Genel_Rapor.xlsx
@@ -191,7 +191,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="52">
+  <borders count="54">
     <border>
       <left/>
       <right/>
@@ -809,11 +809,35 @@
     <border>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1320,6 +1344,13 @@
     <xf numFmtId="0" fontId="15" fillId="6" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="52" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="44" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3435,17 +3466,25 @@
       <c r="BP2" s="7" t="n"/>
     </row>
     <row r="3" ht="31.8" customHeight="1" s="42">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Proje</t>
-        </is>
-      </c>
-      <c r="B3" s="151" t="n"/>
-      <c r="C3" s="152" t="n"/>
+      <c r="B3" s="156" t="n"/>
+      <c r="C3" s="157" t="inlineStr">
+        <is>
+          <t>Proje:</t>
+        </is>
+      </c>
       <c r="D3" s="153" t="n"/>
       <c r="E3" s="153" t="n"/>
       <c r="F3" s="154" t="n"/>
       <c r="G3" s="97" t="inlineStr"/>
+      <c r="H3" s="153" t="n"/>
+      <c r="I3" s="153" t="n"/>
+      <c r="J3" s="153" t="n"/>
+      <c r="K3" s="153" t="n"/>
+      <c r="L3" s="153" t="n"/>
+      <c r="M3" s="153" t="n"/>
+      <c r="N3" s="153" t="n"/>
+      <c r="O3" s="153" t="n"/>
+      <c r="P3" s="154" t="n"/>
     </row>
     <row r="4" ht="20.4" customHeight="1" s="42">
       <c r="B4" s="156" t="n"/>
@@ -3626,7 +3665,7 @@
       <c r="BP6" s="160" t="n"/>
     </row>
     <row r="7" ht="20.4" customHeight="1" s="42" thickBot="1">
-      <c r="B7" s="156" t="n"/>
+      <c r="B7" s="165" t="n"/>
       <c r="C7" s="157" t="inlineStr">
         <is>
           <t>Rapor Gün Sayısı:</t>
@@ -3846,33 +3885,24 @@
       <c r="BP11" s="7" t="n"/>
     </row>
     <row r="12" ht="19.95" customHeight="1" s="42">
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B12" s="190" t="inlineStr">
         <is>
           <t>GRUP FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="C12" s="33" t="n"/>
-      <c r="D12" s="33" t="n"/>
-      <c r="E12" s="33" t="n"/>
-      <c r="F12" s="33" t="n"/>
-      <c r="G12" s="33" t="n"/>
-      <c r="H12" s="33" t="n"/>
-      <c r="I12" s="33" t="n"/>
-      <c r="J12" s="33" t="n"/>
-      <c r="K12" s="33" t="n"/>
-      <c r="L12" s="33" t="n"/>
-      <c r="M12" s="33" t="n"/>
-      <c r="N12" s="33" t="n"/>
-      <c r="O12" s="33" t="n"/>
-      <c r="P12" s="33" t="n"/>
-      <c r="Q12" s="33" t="n"/>
-      <c r="R12" s="33" t="n"/>
-      <c r="S12" s="33" t="n"/>
-      <c r="T12" s="33" t="n"/>
-      <c r="U12" s="33" t="n"/>
-      <c r="V12" s="33" t="n"/>
-      <c r="W12" s="33" t="n"/>
-      <c r="X12" s="33" t="n"/>
+      <c r="D12" s="191" t="n"/>
+      <c r="E12" s="192" t="n"/>
+      <c r="G12" s="191" t="n"/>
+      <c r="H12" s="192" t="n"/>
+      <c r="J12" s="191" t="n"/>
+      <c r="K12" s="192" t="n"/>
+      <c r="N12" s="191" t="n"/>
+      <c r="O12" s="192" t="n"/>
+      <c r="Q12" s="191" t="n"/>
+      <c r="R12" s="192" t="n"/>
+      <c r="U12" s="191" t="n"/>
+      <c r="V12" s="192" t="n"/>
+      <c r="X12" s="191" t="n"/>
       <c r="Y12" s="33" t="n"/>
       <c r="Z12" s="33" t="n"/>
       <c r="AA12" s="34" t="inlineStr">
@@ -3880,108 +3910,32 @@
           <t>FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="AB12" s="33" t="n"/>
-      <c r="AC12" s="33" t="n"/>
-      <c r="AD12" s="33" t="n"/>
-      <c r="AE12" s="33" t="n"/>
-      <c r="AF12" s="33" t="n"/>
-      <c r="AG12" s="33" t="n"/>
-      <c r="AH12" s="33" t="n"/>
-      <c r="AI12" s="33" t="n"/>
-      <c r="AJ12" s="33" t="n"/>
       <c r="AK12" s="33" t="n"/>
-      <c r="AL12" s="33" t="n"/>
-      <c r="AM12" s="33" t="n"/>
-      <c r="AN12" s="33" t="n"/>
       <c r="AO12" s="33" t="n"/>
       <c r="AP12" s="34" t="inlineStr">
         <is>
           <t>FREKANS SAPMALARI</t>
         </is>
       </c>
-      <c r="AQ12" s="33" t="n"/>
-      <c r="AR12" s="33" t="n"/>
-      <c r="AS12" s="33" t="n"/>
-      <c r="AT12" s="33" t="n"/>
-      <c r="AU12" s="33" t="n"/>
-      <c r="AV12" s="33" t="n"/>
-      <c r="AW12" s="33" t="n"/>
-      <c r="AX12" s="33" t="n"/>
-      <c r="AY12" s="33" t="n"/>
       <c r="AZ12" s="33" t="n"/>
-      <c r="BA12" s="33" t="n"/>
-      <c r="BB12" s="33" t="n"/>
       <c r="BC12" s="33" t="n"/>
       <c r="BD12" s="34" t="inlineStr">
         <is>
           <t>KAYIP FREKANS GÖSTERGELERİ</t>
         </is>
       </c>
-      <c r="BE12" s="33" t="n"/>
-      <c r="BF12" s="33" t="n"/>
-      <c r="BG12" s="33" t="n"/>
-      <c r="BH12" s="33" t="n"/>
-      <c r="BI12" s="33" t="n"/>
-      <c r="BJ12" s="33" t="n"/>
-      <c r="BK12" s="33" t="n"/>
-      <c r="BL12" s="33" t="n"/>
-      <c r="BM12" s="33" t="n"/>
       <c r="BN12" s="33" t="n"/>
-      <c r="BO12" s="33" t="n"/>
       <c r="BP12" s="15" t="n"/>
     </row>
     <row r="13" ht="19.95" customHeight="1" s="42">
-      <c r="B13" s="84" t="inlineStr">
-        <is>
-          <t>GRUP TANIMI</t>
-        </is>
-      </c>
-      <c r="C13" s="175" t="n"/>
-      <c r="D13" s="176" t="n"/>
-      <c r="E13" s="85" t="inlineStr">
-        <is>
-          <t>HEDEF FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="F13" s="175" t="n"/>
-      <c r="G13" s="176" t="n"/>
-      <c r="H13" s="85" t="inlineStr">
-        <is>
-          <t>TAMAMLANMIŞ FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="I13" s="175" t="n"/>
-      <c r="J13" s="176" t="n"/>
-      <c r="K13" s="85" t="inlineStr">
-        <is>
-          <t>ZAMANINDA GERÇEKLEŞEN İŞLEM ORANI</t>
-        </is>
-      </c>
-      <c r="L13" s="175" t="n"/>
-      <c r="M13" s="175" t="n"/>
-      <c r="N13" s="176" t="n"/>
-      <c r="O13" s="85" t="inlineStr">
-        <is>
-          <t>SAPMA FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="P13" s="175" t="n"/>
-      <c r="Q13" s="176" t="n"/>
-      <c r="R13" s="85" t="inlineStr">
-        <is>
-          <t>KAYIP FREKANS SAYISI</t>
-        </is>
-      </c>
-      <c r="S13" s="175" t="n"/>
-      <c r="T13" s="175" t="n"/>
-      <c r="U13" s="176" t="n"/>
-      <c r="V13" s="177" t="inlineStr">
-        <is>
-          <t>GENEL ORAN</t>
-        </is>
-      </c>
-      <c r="W13" s="175" t="n"/>
-      <c r="X13" s="176" t="n"/>
+      <c r="B13" s="9" t="n"/>
+      <c r="D13" s="191" t="n"/>
+      <c r="G13" s="191" t="n"/>
+      <c r="J13" s="191" t="n"/>
+      <c r="N13" s="191" t="n"/>
+      <c r="Q13" s="191" t="n"/>
+      <c r="U13" s="191" t="n"/>
+      <c r="X13" s="191" t="n"/>
       <c r="AA13" s="53" t="inlineStr">
         <is>
           <t>Toplam Frekans Sayısı</t>
@@ -4042,27 +3996,27 @@
       </c>
     </row>
     <row r="14" ht="22.2" customHeight="1" s="42">
-      <c r="B14" s="178" t="n"/>
+      <c r="B14" s="193" t="n"/>
       <c r="C14" s="179" t="n"/>
       <c r="D14" s="180" t="n"/>
-      <c r="E14" s="181" t="n"/>
+      <c r="E14" s="194" t="n"/>
       <c r="F14" s="179" t="n"/>
       <c r="G14" s="180" t="n"/>
-      <c r="H14" s="181" t="n"/>
+      <c r="H14" s="194" t="n"/>
       <c r="I14" s="179" t="n"/>
       <c r="J14" s="180" t="n"/>
-      <c r="K14" s="181" t="n"/>
+      <c r="K14" s="194" t="n"/>
       <c r="L14" s="179" t="n"/>
       <c r="M14" s="179" t="n"/>
       <c r="N14" s="180" t="n"/>
-      <c r="O14" s="181" t="n"/>
+      <c r="O14" s="194" t="n"/>
       <c r="P14" s="179" t="n"/>
       <c r="Q14" s="180" t="n"/>
-      <c r="R14" s="181" t="n"/>
+      <c r="R14" s="194" t="n"/>
       <c r="S14" s="179" t="n"/>
       <c r="T14" s="179" t="n"/>
       <c r="U14" s="180" t="n"/>
-      <c r="V14" s="179" t="n"/>
+      <c r="V14" s="180" t="n"/>
       <c r="W14" s="179" t="n"/>
       <c r="X14" s="180" t="n"/>
       <c r="AA14" s="53" t="inlineStr">
@@ -5082,6 +5036,11 @@
           <t>DURUM</t>
         </is>
       </c>
+      <c r="G2" s="189" t="inlineStr">
+        <is>
+          <t>KAYIP NEDENİ</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="21.6" customHeight="1" s="42">
       <c r="A3" s="183" t="inlineStr">
@@ -5093,11 +5052,7 @@
         <f>COUNTA(A4:A5000)</f>
         <v/>
       </c>
-      <c r="G3" s="189" t="inlineStr">
-        <is>
-          <t>KAYIP NEDENİ</t>
-        </is>
-      </c>
+      <c r="G3" s="189" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="35" t="n">

</xml_diff>